<commit_message>
some changes in app and review files
</commit_message>
<xml_diff>
--- a/review/review_ar.xlsx
+++ b/review/review_ar.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,13 +34,22 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -60,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -71,13 +80,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -445,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -558,64 +573,78 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>• Rows marked 🌍 name the asker's nationality. Check that this sounds right.</t>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>• IMPORTANT: Mixing in German words (Ausbildung, Anmeldung) is fine if people really do that. But if there is an expression in your language, use it preferably.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>• Everyday wording is better than formal or legal wording.</t>
+          <t>• Rows marked 🌍 name the asker's nationality. Check that this sounds right.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>• This set is written in Modern Standard Arabic on purpose: it is the baseline. Please keep it standard Arabic. A separate file covers the Syrian dialect.</t>
+          <t>• Everyday wording is better than formal or legal wording.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>• This set is written in Modern Standard Arabic on purpose: it is the baseline. Please keep it standard Arabic. A separate file covers the Syrian dialect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>• Some questions use the masculine form (for example مواطن). If a neutral or feminine form would be more natural, say so in Comment.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr"/>
-    </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Please don't change the topic of a question or the numbers in it (for example 48,000 euros, 32 years old).</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>When you are done, send this file back. Thank you!</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
-    </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>هذه الجمل مسودة أولى كتبها نموذج ذكاء اصطناعي (Claude Opus 5.5)، وقد تحتوي على أخطاء أو صياغات غير طبيعية، فلا تتردد في تصحيحها كما تكتبها أنت.</t>
-        </is>
-      </c>
+      <c r="A27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
+          <t>هذه الجمل مسودة أولى كتبها نموذج ذكاء اصطناعي (Claude Opus 5.5)، وقد تحتوي على أخطاء أو صياغات غير طبيعية، فلا تتردد في تصحيحها كما تكتبها أنت.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
           <t>ملخص: في ورقة Questions، اقرأ الجملة الإنجليزية ثم الترجمة العربية. إذا كانت صحيحة وطبيعية، اختر ✓ في عمود OK? ولا تكتب شيئاً آخر. إذا كان فيها خطأ أو كانت غير طبيعية، اكتب صيغتك في عمود Correction. لا تغيّر المعنى، صحّح اللغة فقط، وأبقِ الأسئلة بالفصحى. شكراً لك!</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>مهم: يمكن استخدام كلمات ألمانية (مثل Ausbildung أو Anmeldung) إذا كان الناس يستخدمونها فعلاً، لكن إذا وُجد تعبير بالعربية فالأفضل استخدامه.</t>
         </is>
       </c>
     </row>
@@ -643,37 +672,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>Arabic</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>OK?</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>Correction</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="8" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
@@ -693,13 +722,13 @@
           <t>🌍 I'm American. Once I finish my master's degree in Germany, can I get a work visa?</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>أنا أمريكي. هل يمكنني الحصول على تأشيرة عمل بعد أن أنهي الماجستير في ألمانيا؟</t>
         </is>
       </c>
       <c r="E2" s="2" t="n"/>
-      <c r="F2" s="5" t="n"/>
+      <c r="F2" s="6" t="n"/>
       <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
@@ -716,13 +745,13 @@
           <t>🌍 What do Nigerian citizens have to do to work in Germany?</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>ما الذي يجب على المواطنين النيجيريين فعله للعمل في ألمانيا؟</t>
         </is>
       </c>
       <c r="E3" s="2" t="n"/>
-      <c r="F3" s="5" t="n"/>
+      <c r="F3" s="6" t="n"/>
       <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
@@ -739,13 +768,13 @@
           <t>🌍 I'm moving from Italy to Germany. Do I have to do the Anmeldung?</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>سأنتقل من إيطاليا إلى ألمانيا. هل يجب أن أقوم بتسجيل السكن؟</t>
         </is>
       </c>
       <c r="E4" s="2" t="n"/>
-      <c r="F4" s="5" t="n"/>
+      <c r="F4" s="6" t="n"/>
       <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
@@ -762,13 +791,13 @@
           <t>🌍 Can Polish citizens live in Germany without a visa and without doing the Anmeldung?</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>هل يمكن للمواطنين البولنديين العيش في ألمانيا دون تأشيرة ودون تسجيل السكن؟</t>
         </is>
       </c>
       <c r="E5" s="2" t="n"/>
-      <c r="F5" s="5" t="n"/>
+      <c r="F5" s="6" t="n"/>
       <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
@@ -785,13 +814,13 @@
           <t>🌍 I'm Syrian and I'm here as a refugee. What money can I receive?</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>أنا سوري وموجود هنا كلاجئ. ما المساعدات المالية التي يمكنني الحصول عليها؟</t>
         </is>
       </c>
       <c r="E6" s="2" t="n"/>
-      <c r="F6" s="5" t="n"/>
+      <c r="F6" s="6" t="n"/>
       <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
@@ -808,13 +837,13 @@
           <t>🌍 I'm coming to Germany from India. Do I need a visa?</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>سأدخل ألمانيا قادماً من الهند. هل أحتاج إلى تأشيرة؟</t>
         </is>
       </c>
       <c r="E7" s="2" t="n"/>
-      <c r="F7" s="5" t="n"/>
+      <c r="F7" s="6" t="n"/>
       <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
@@ -831,13 +860,13 @@
           <t>🌍 Can someone with dual citizenship get permanent residence in Germany? The countries are Brazil and Australia.</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>هل يمكن لمزدوجي الجنسية الحصول على الإقامة الدائمة في ألمانيا؟ الجنسيتان هما البرازيلية والأسترالية.</t>
         </is>
       </c>
       <c r="E8" s="2" t="n"/>
-      <c r="F8" s="5" t="n"/>
+      <c r="F8" s="6" t="n"/>
       <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
@@ -854,13 +883,13 @@
           <t>Citizens of which countries can enter Germany without a visa and stay for more than two months?</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>ما الجنسيات التي يمكن لأصحابها دخول ألمانيا دون تأشيرة والبقاء فيها أكثر من شهرين؟</t>
         </is>
       </c>
       <c r="E9" s="2" t="n"/>
-      <c r="F9" s="5" t="n"/>
+      <c r="F9" s="6" t="n"/>
       <c r="G9" s="2" t="n"/>
     </row>
     <row r="10">
@@ -877,13 +906,13 @@
           <t>Does Germany have a visa for freelancers?</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>هل يوجد في ألمانيا تأشيرة خاصة بالعمل الحر (الفريلانسر)؟</t>
         </is>
       </c>
       <c r="E10" s="2" t="n"/>
-      <c r="F10" s="5" t="n"/>
+      <c r="F10" s="6" t="n"/>
       <c r="G10" s="2" t="n"/>
     </row>
     <row r="11">
@@ -900,13 +929,13 @@
           <t>Can people from non-EU countries also join the artists' social insurance?</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>هل يمكن للأشخاص من دول خارج الاتحاد الأوروبي أيضاً الانضمام إلى التأمين الاجتماعي للفنانين؟</t>
         </is>
       </c>
       <c r="E11" s="2" t="n"/>
-      <c r="F11" s="5" t="n"/>
+      <c r="F11" s="6" t="n"/>
       <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
@@ -923,13 +952,13 @@
           <t>After graduating I got the 18-month job-seeker residence permit. If I don't find a job within 18 months, do I have to leave Germany? Can it be extended?</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>بعد التخرج حصلت على تصريح إقامة للبحث عن عمل لمدة 18 شهراً. إذا لم أجد عملاً خلال 18 شهراً، فهل يجب أن أغادر ألمانيا؟ وهل يمكن تمديده؟</t>
         </is>
       </c>
       <c r="E12" s="2" t="n"/>
-      <c r="F12" s="5" t="n"/>
+      <c r="F12" s="6" t="n"/>
       <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
@@ -946,13 +975,13 @@
           <t>🌍 I'm South Korean and stayed in Germany visa-free for two and a half months. If I go back home and then come back, can I stay again for less than three months?</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>أنا كوري جنوبي وبقيت في ألمانيا شهرين ونصفاً دون تأشيرة. إذا عدت إلى بلدي ثم رجعت، فهل يمكنني البقاء مرة أخرى أقل من ثلاثة أشهر؟</t>
         </is>
       </c>
       <c r="E13" s="2" t="n"/>
-      <c r="F13" s="5" t="n"/>
+      <c r="F13" s="6" t="n"/>
       <c r="G13" s="2" t="n"/>
     </row>
     <row r="14">
@@ -969,13 +998,13 @@
           <t>Can non-EU students work in Germany while they study? How much are they allowed to work?</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>هل يمكن للطلاب الأجانب من خارج الاتحاد الأوروبي العمل في ألمانيا أثناء دراستهم؟ وما مقدار العمل المسموح لهم به؟</t>
         </is>
       </c>
       <c r="E14" s="2" t="n"/>
-      <c r="F14" s="5" t="n"/>
+      <c r="F14" s="6" t="n"/>
       <c r="G14" s="2" t="n"/>
     </row>
     <row r="15">
@@ -992,13 +1021,13 @@
           <t>🌍 I'm Mexican. If I get German citizenship, do I have to give up my Mexican citizenship?</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>أنا مكسيكي. إذا حصلت على الجنسية الألمانية، فهل يجب أن أتخلى عن جنسيتي المكسيكية؟</t>
         </is>
       </c>
       <c r="E15" s="2" t="n"/>
-      <c r="F15" s="5" t="n"/>
+      <c r="F15" s="6" t="n"/>
       <c r="G15" s="2" t="n"/>
     </row>
     <row r="16">
@@ -1015,13 +1044,13 @@
           <t>How many years do I have to live in Germany before I can get an EU Blue Card?</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>كم سنة يجب أن أعيش في ألمانيا قبل أن أتمكن من الحصول على البطاقة الزرقاء؟</t>
         </is>
       </c>
       <c r="E16" s="2" t="n"/>
-      <c r="F16" s="5" t="n"/>
+      <c r="F16" s="6" t="n"/>
       <c r="G16" s="2" t="n"/>
     </row>
     <row r="17">
@@ -1038,13 +1067,13 @@
           <t>🌍 I'm Vietnamese. What residence permit do I need to do an Ausbildung in Germany, and what are the conditions?</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>أنا فيتنامي. ما تصريح الإقامة الذي أحتاجه لعمل أوسبيلدونغ في ألمانيا، وما شروطه؟</t>
         </is>
       </c>
       <c r="E17" s="2" t="n"/>
-      <c r="F17" s="5" t="n"/>
+      <c r="F17" s="6" t="n"/>
       <c r="G17" s="2" t="n"/>
     </row>
     <row r="18">
@@ -1061,13 +1090,13 @@
           <t>How long after getting an EU Blue Card can I get a permanent settlement permit?</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>بعد كم من الوقت من حصولي على البطاقة الزرقاء يمكنني الحصول على الإقامة الدائمة؟</t>
         </is>
       </c>
       <c r="E18" s="2" t="n"/>
-      <c r="F18" s="5" t="n"/>
+      <c r="F18" s="6" t="n"/>
       <c r="G18" s="2" t="n"/>
     </row>
     <row r="19">
@@ -1084,13 +1113,13 @@
           <t>I don't have a university degree, only work experience in IT. Can I get an EU Blue Card?</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>ليست لدي شهادة جامعية، بل خبرة عملية في مجال تكنولوجيا المعلومات فقط. هل يمكنني الحصول على البطاقة الزرقاء الأوروبية؟</t>
         </is>
       </c>
       <c r="E19" s="2" t="n"/>
-      <c r="F19" s="5" t="n"/>
+      <c r="F19" s="6" t="n"/>
       <c r="G19" s="2" t="n"/>
     </row>
     <row r="20">
@@ -1107,13 +1136,13 @@
           <t>Can I have a side job while I'm doing my Ausbildung?</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>هل يمكنني العمل في وظيفة جانبية أثناء الأوسبيلدونغ؟</t>
         </is>
       </c>
       <c r="E20" s="2" t="n"/>
-      <c r="F20" s="5" t="n"/>
+      <c r="F20" s="6" t="n"/>
       <c r="G20" s="2" t="n"/>
     </row>
     <row r="21">
@@ -1130,13 +1159,13 @@
           <t>If a German company wants to bring in a foreign employee quickly, is there a way to speed up the process?</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>إذا أرادت شركة ألمانية استقدام موظف أجنبي بسرعة، فهل هناك طريقة لتسريع الإجراءات؟</t>
         </is>
       </c>
       <c r="E21" s="2" t="n"/>
-      <c r="F21" s="5" t="n"/>
+      <c r="F21" s="6" t="n"/>
       <c r="G21" s="2" t="n"/>
     </row>
     <row r="22">
@@ -1153,13 +1182,13 @@
           <t>If I'm working on an employment residence permit and quit my job earlier than planned, do I have to tell the immigration office?</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>إذا كنت أعمل بتصريح إقامة لغرض العمل وتركت وظيفتي قبل الموعد المخطط له، فهل يجب أن أبلغ دائرة الأجانب؟</t>
         </is>
       </c>
       <c r="E22" s="2" t="n"/>
-      <c r="F22" s="5" t="n"/>
+      <c r="F22" s="6" t="n"/>
       <c r="G22" s="2" t="n"/>
     </row>
     <row r="23">
@@ -1176,13 +1205,13 @@
           <t>What conditions do I have to meet to get a regular settlement permit without a Blue Card?</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>ما الشروط التي يجب أن أستوفيها للحصول على تصريح إقامة دائمة عادي دون البطاقة الزرقاء؟</t>
         </is>
       </c>
       <c r="E23" s="2" t="n"/>
-      <c r="F23" s="5" t="n"/>
+      <c r="F23" s="6" t="n"/>
       <c r="G23" s="2" t="n"/>
     </row>
     <row r="24">
@@ -1199,13 +1228,13 @@
           <t>🌍 I'm a student from Kenya. Do I have to join the public health insurance in Germany?</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>أنا طالب من كينيا. هل يجب عليّ الاشتراك في التأمين الصحي الحكومي في ألمانيا؟</t>
         </is>
       </c>
       <c r="E24" s="2" t="n"/>
-      <c r="F24" s="5" t="n"/>
+      <c r="F24" s="6" t="n"/>
       <c r="G24" s="2" t="n"/>
     </row>
     <row r="25">
@@ -1222,13 +1251,13 @@
           <t>🌍 I'm from Colombia. What are the requirements for working as an au pair in Germany?</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>أنا من كولومبيا. ما شروط العمل كأوبير في ألمانيا؟</t>
         </is>
       </c>
       <c r="E25" s="2" t="n"/>
-      <c r="F25" s="5" t="n"/>
+      <c r="F25" s="6" t="n"/>
       <c r="G25" s="2" t="n"/>
     </row>
     <row r="26">
@@ -1245,13 +1274,13 @@
           <t>I'm still enrolled at university but I've found a full-time job. Can I switch to a work residence permit before I graduate?</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>ما زلت مسجلاً في الجامعة لكنني وجدت وظيفة بدوام كامل. هل يمكنني التحول إلى تصريح إقامة لغرض العمل قبل التخرج؟</t>
         </is>
       </c>
       <c r="E26" s="2" t="n"/>
-      <c r="F26" s="5" t="n"/>
+      <c r="F26" s="6" t="n"/>
       <c r="G26" s="2" t="n"/>
     </row>
     <row r="27">
@@ -1268,13 +1297,13 @@
           <t>What conditions do I need to meet to get an Opportunity Card?</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>ما الشروط التي يجب أن أستوفيها للحصول على بطاقة الفرص؟</t>
         </is>
       </c>
       <c r="E27" s="2" t="n"/>
-      <c r="F27" s="5" t="n"/>
+      <c r="F27" s="6" t="n"/>
       <c r="G27" s="2" t="n"/>
     </row>
     <row r="28">
@@ -1291,13 +1320,13 @@
           <t>🌍 Can South Korean citizens get a work visa for Germany without a university degree?</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>هل يمكن للمواطنين الكوريين الجنوبيين الحصول على تأشيرة عمل في ألمانيا دون شهادة جامعية؟</t>
         </is>
       </c>
       <c r="E28" s="2" t="n"/>
-      <c r="F28" s="5" t="n"/>
+      <c r="F28" s="6" t="n"/>
       <c r="G28" s="2" t="n"/>
     </row>
     <row r="29">
@@ -1314,13 +1343,13 @@
           <t>What does someone who completed vocational training abroad need to get a work residence permit in Germany?</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>ما الذي يحتاجه شخص أكمل تدريبه المهني في الخارج للحصول على تصريح إقامة لغرض العمل في ألمانيا؟</t>
         </is>
       </c>
       <c r="E29" s="2" t="n"/>
-      <c r="F29" s="5" t="n"/>
+      <c r="F29" s="6" t="n"/>
       <c r="G29" s="2" t="n"/>
     </row>
     <row r="30">
@@ -1337,13 +1366,13 @@
           <t>🌍 I'm Austrian and live in Germany. When I move back home, do I have to do the Abmeldung?</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>أنا نمساوي وأعيش في ألمانيا. عندما أعود إلى بلدي، هل يجب أن ألغي تسجيل السكن؟</t>
         </is>
       </c>
       <c r="E30" s="2" t="n"/>
-      <c r="F30" s="5" t="n"/>
+      <c r="F30" s="6" t="n"/>
       <c r="G30" s="2" t="n"/>
     </row>
     <row r="31">
@@ -1360,13 +1389,13 @@
           <t>🌍 I'm Serbian. I have no degree and no qualification recognised in Germany, but long practical work experience. Can I work in Germany?</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>أنا صربي. ليست لدي شهادة ولا مؤهل معترف به في ألمانيا، لكن لدي خبرة عملية طويلة. هل يمكنني العمل في ألمانيا؟</t>
         </is>
       </c>
       <c r="E31" s="2" t="n"/>
-      <c r="F31" s="5" t="n"/>
+      <c r="F31" s="6" t="n"/>
       <c r="G31" s="2" t="n"/>
     </row>
     <row r="32">
@@ -1383,13 +1412,13 @@
           <t>If I work on a regular skilled-worker residence permit rather than a Blue Card, after how many years can I get a settlement permit?</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>إذا عملت بتصريح إقامة عادي للعمالة الماهرة بدلاً من البطاقة الزرقاء، فبعد كم سنة يمكنني الحصول على تصريح الإقامة الدائمة؟</t>
         </is>
       </c>
       <c r="E32" s="2" t="n"/>
-      <c r="F32" s="5" t="n"/>
+      <c r="F32" s="6" t="n"/>
       <c r="G32" s="2" t="n"/>
     </row>
     <row r="33">
@@ -1406,13 +1435,13 @@
           <t>What does the Federal Employment Agency check when a company hires a foreign worker?</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>ما الذي تفحصه الوكالة الاتحادية للعمل عندما توظف شركة عاملاً أجنبياً؟</t>
         </is>
       </c>
       <c r="E33" s="2" t="n"/>
-      <c r="F33" s="5" t="n"/>
+      <c r="F33" s="6" t="n"/>
       <c r="G33" s="2" t="n"/>
     </row>
     <row r="34">
@@ -1429,13 +1458,13 @@
           <t>🌍 I'm a nurse from the Philippines, and my qualification was only partly recognised in Germany. Can I stay and work in Germany while I make up for what's missing?</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>أنا ممرض من الفلبين، واعتُرف بمؤهلي في ألمانيا اعترافاً جزئياً فقط. هل يمكنني البقاء والعمل في ألمانيا ريثما أستكمل ما ينقصني؟</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
-      <c r="F34" s="5" t="n"/>
+      <c r="F34" s="6" t="n"/>
       <c r="G34" s="2" t="n"/>
     </row>
     <row r="35">
@@ -1452,13 +1481,13 @@
           <t>Even if I meet all the requirements, on what grounds can a work residence permit still be refused?</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>حتى لو استوفيت جميع الشروط، ما الأسباب التي قد يُرفض بسببها تصريح الإقامة لغرض العمل؟</t>
         </is>
       </c>
       <c r="E35" s="2" t="n"/>
-      <c r="F35" s="5" t="n"/>
+      <c r="F35" s="6" t="n"/>
       <c r="G35" s="2" t="n"/>
     </row>
     <row r="36">
@@ -1475,13 +1504,13 @@
           <t>🌍 Can a Turkish citizen come to Germany for a seasonal job that lasts only a few months, like a farm harvest?</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>هل يمكن لمواطن تركي القدوم إلى ألمانيا من أجل عمل موسمي يستمر بضعة أشهر فقط، مثل حصاد المزارع؟</t>
         </is>
       </c>
       <c r="E36" s="2" t="n"/>
-      <c r="F36" s="5" t="n"/>
+      <c r="F36" s="6" t="n"/>
       <c r="G36" s="2" t="n"/>
     </row>
     <row r="37">
@@ -1498,13 +1527,13 @@
           <t>🌍 I'm Portuguese and work at the head office of a Spanish company. If I'm transferred to the German branch, what residence permit do I need?</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>أنا برتغالي وأعمل في المقر الرئيسي لشركة إسبانية. إذا نُقلت إلى فرع الشركة في ألمانيا، فما تصريح الإقامة الذي يجب أن أحصل عليه؟</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
-      <c r="F37" s="5" t="n"/>
+      <c r="F37" s="6" t="n"/>
       <c r="G37" s="2" t="n"/>
     </row>
     <row r="38">
@@ -1521,13 +1550,13 @@
           <t>Whether they are EU or non-EU citizens, do people in Germany have to pay social insurance or pension insurance contributions?</t>
         </is>
       </c>
-      <c r="D38" s="5" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>سواء كانوا مواطنين من الاتحاد الأوروبي أو من خارجه، هل يجب على الناس في ألمانيا دفع اشتراكات التأمين الاجتماعي أو تأمين التقاعد؟</t>
         </is>
       </c>
       <c r="E38" s="2" t="n"/>
-      <c r="F38" s="5" t="n"/>
+      <c r="F38" s="6" t="n"/>
       <c r="G38" s="2" t="n"/>
     </row>
     <row r="39">
@@ -1544,13 +1573,13 @@
           <t>Do EU citizens who move to Germany not have to do their Anmeldung?</t>
         </is>
       </c>
-      <c r="D39" s="5" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>أليس على مواطني الاتحاد الأوروبي الذين ينتقلون إلى ألمانيا تسجيل السكن؟</t>
         </is>
       </c>
       <c r="E39" s="2" t="n"/>
-      <c r="F39" s="5" t="n"/>
+      <c r="F39" s="6" t="n"/>
       <c r="G39" s="2" t="n"/>
     </row>
     <row r="40">
@@ -1567,13 +1596,13 @@
           <t>🌍 I'm a Syrian citizen and applied for the October semester, but I haven't heard back yet. The semester starts in a month. Will I be able to get a visa?</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>أنا مواطن سوري وتقدمت للفصل الدراسي الذي يبدأ في أكتوبر، لكنني لم أتلقَّ رداً بعد. يبدأ الفصل بعد شهر. هل سأتمكن من الحصول على تأشيرة؟</t>
         </is>
       </c>
       <c r="E40" s="2" t="n"/>
-      <c r="F40" s="5" t="n"/>
+      <c r="F40" s="6" t="n"/>
       <c r="G40" s="2" t="n"/>
     </row>
     <row r="41">
@@ -1590,13 +1619,13 @@
           <t>How many years do I have to live in Germany before I can get German citizenship?</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>كم سنة يجب أن أعيش في ألمانيا قبل أن أتمكن من الحصول على الجنسية الألمانية؟</t>
         </is>
       </c>
       <c r="E41" s="2" t="n"/>
-      <c r="F41" s="5" t="n"/>
+      <c r="F41" s="6" t="n"/>
       <c r="G41" s="2" t="n"/>
     </row>
     <row r="42">
@@ -1613,13 +1642,13 @@
           <t>🌍 I'm 32, Chinese, and have a bachelor's degree in computer science. I've been offered a salary of 48,000 euros. Will I get a Blue Card?</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>عمري 32 عاماً، وأنا صيني، وأحمل درجة البكالوريوس في هندسة الحاسوب. تلقيت عرضاً براتب 48,000 يورو. هل سأحصل على البطاقة الزرقاء؟</t>
         </is>
       </c>
       <c r="E42" s="2" t="n"/>
-      <c r="F42" s="5" t="n"/>
+      <c r="F42" s="6" t="n"/>
       <c r="G42" s="2" t="n"/>
     </row>
     <row r="43">
@@ -1636,13 +1665,13 @@
           <t>🌍 I'm Japanese, and the immigration office refused to extend my work residence permit. Is that decision unlawful? Would I win if I sued?</t>
         </is>
       </c>
-      <c r="D43" s="5" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>أنا ياباني، ورفضت دائرة الأجانب تمديد تصريح إقامتي لغرض العمل. هل هذا القرار غير قانوني؟ هل سأكسب القضية إذا رفعت دعوى؟</t>
         </is>
       </c>
       <c r="E43" s="2" t="n"/>
-      <c r="F43" s="5" t="n"/>
+      <c r="F43" s="6" t="n"/>
       <c r="G43" s="2" t="n"/>
     </row>
     <row r="44">
@@ -1659,13 +1688,13 @@
           <t>Can I work as a freelancer in Germany? If so, do I have to register somewhere first?</t>
         </is>
       </c>
-      <c r="D44" s="5" t="inlineStr">
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>هل يمكنني العمل كفريلانسر في ألمانيا؟ وإذا كان ذلك ممكناً، هل يجب أن أسجل في مكان ما أولاً؟</t>
         </is>
       </c>
       <c r="E44" s="2" t="n"/>
-      <c r="F44" s="5" t="n"/>
+      <c r="F44" s="6" t="n"/>
       <c r="G44" s="2" t="n"/>
     </row>
     <row r="45">
@@ -1682,13 +1711,13 @@
           <t>Do Werkstudents and HiWis have to pay into the pension insurance? Or does the company or university take care of it?</t>
         </is>
       </c>
-      <c r="D45" s="5" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>هل يجب على طلاب الـ Werkstudent والـ HiWi دفع اشتراكات تأمين التقاعد؟ أم أن الشركة أو الجامعة تتولى ذلك؟</t>
         </is>
       </c>
       <c r="E45" s="2" t="n"/>
-      <c r="F45" s="5" t="n"/>
+      <c r="F45" s="6" t="n"/>
       <c r="G45" s="2" t="n"/>
     </row>
     <row r="46">
@@ -1705,13 +1734,13 @@
           <t>Can I get back the taxes I paid when I go back home?</t>
         </is>
       </c>
-      <c r="D46" s="5" t="inlineStr">
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>هل يمكنني استرداد الضرائب التي دفعتها عند عودتي إلى بلدي؟</t>
         </is>
       </c>
       <c r="E46" s="2" t="n"/>
-      <c r="F46" s="5" t="n"/>
+      <c r="F46" s="6" t="n"/>
       <c r="G46" s="2" t="n"/>
     </row>
     <row r="47">
@@ -1728,13 +1757,13 @@
           <t>🌍 I'm Spanish. How many months do I have to live in Germany before I have to pay tax here?</t>
         </is>
       </c>
-      <c r="D47" s="5" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>أنا إسباني. كم شهراً يجب أن أعيش في ألمانيا حتى يصبح عليّ دفع الضرائب فيها؟</t>
         </is>
       </c>
       <c r="E47" s="2" t="n"/>
-      <c r="F47" s="5" t="n"/>
+      <c r="F47" s="6" t="n"/>
       <c r="G47" s="2" t="n"/>
     </row>
     <row r="48">
@@ -1751,13 +1780,13 @@
           <t>🌍 My spouse lives in Canada. Can we be taxed jointly in Germany?</t>
         </is>
       </c>
-      <c r="D48" s="5" t="inlineStr">
+      <c r="D48" s="6" t="inlineStr">
         <is>
           <t>زوجتي أو زوجي يعيش في كندا. هل يمكننا الخضوع للتقييم الضريبي المشترك في ألمانيا؟</t>
         </is>
       </c>
       <c r="E48" s="2" t="n"/>
-      <c r="F48" s="5" t="n"/>
+      <c r="F48" s="6" t="n"/>
       <c r="G48" s="2" t="n"/>
     </row>
     <row r="49">
@@ -1774,13 +1803,13 @@
           <t>🌍 I'm a South African citizen. Can I get Kindergeld in Germany?</t>
         </is>
       </c>
-      <c r="D49" s="5" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>أنا مواطن من جنوب أفريقيا. هل يمكنني الحصول على الكيندرغيلد في ألمانيا؟</t>
         </is>
       </c>
       <c r="E49" s="2" t="n"/>
-      <c r="F49" s="5" t="n"/>
+      <c r="F49" s="6" t="n"/>
       <c r="G49" s="2" t="n"/>
     </row>
     <row r="50">
@@ -1797,13 +1826,13 @@
           <t>I also have income in Korea. Do I have to pay tax on it in both countries?</t>
         </is>
       </c>
-      <c r="D50" s="5" t="inlineStr">
+      <c r="D50" s="6" t="inlineStr">
         <is>
           <t>لدي دخل في كوريا الجنوبية أيضاً. هل يجب أن أدفع الضرائب عليه في البلدين؟</t>
         </is>
       </c>
       <c r="E50" s="2" t="n"/>
-      <c r="F50" s="5" t="n"/>
+      <c r="F50" s="6" t="n"/>
       <c r="G50" s="2" t="n"/>
     </row>
     <row r="51">
@@ -1820,13 +1849,13 @@
           <t>When I first come to Germany, how do I get a Steuer-ID?</t>
         </is>
       </c>
-      <c r="D51" s="5" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>عندما أصل إلى ألمانيا لأول مرة، كيف أحصل على الرقم الضريبي؟</t>
         </is>
       </c>
       <c r="E51" s="2" t="n"/>
-      <c r="F51" s="5" t="n"/>
+      <c r="F51" s="6" t="n"/>
       <c r="G51" s="2" t="n"/>
     </row>
     <row r="52">
@@ -1843,13 +1872,13 @@
           <t>Is the money I earn from a Minijob taxed?</t>
         </is>
       </c>
-      <c r="D52" s="5" t="inlineStr">
+      <c r="D52" s="6" t="inlineStr">
         <is>
           <t>هل تُفرض ضريبة على المال الذي أكسبه من الميني جوب؟</t>
         </is>
       </c>
       <c r="E52" s="2" t="n"/>
-      <c r="F52" s="5" t="n"/>
+      <c r="F52" s="6" t="n"/>
       <c r="G52" s="2" t="n"/>
     </row>
     <row r="53">
@@ -1866,13 +1895,13 @@
           <t>If I don't pay into the pension insurance, can I still get permanent residence?</t>
         </is>
       </c>
-      <c r="D53" s="5" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>إذا لم أدفع اشتراكات تأمين التقاعد، هل لن أتمكن من الحصول على الإقامة الدائمة؟</t>
         </is>
       </c>
       <c r="E53" s="2" t="n"/>
-      <c r="F53" s="5" t="n"/>
+      <c r="F53" s="6" t="n"/>
       <c r="G53" s="2" t="n"/>
     </row>
     <row r="54">
@@ -1889,13 +1918,13 @@
           <t>Do foreign students also have to file a tax return? If so, what is the deadline?</t>
         </is>
       </c>
-      <c r="D54" s="5" t="inlineStr">
+      <c r="D54" s="6" t="inlineStr">
         <is>
           <t>هل يجب على الطلاب الأجانب أيضاً تقديم إقرار ضريبي؟ وإذا كان كذلك، فما هو الموعد النهائي؟</t>
         </is>
       </c>
       <c r="E54" s="2" t="n"/>
-      <c r="F54" s="5" t="n"/>
+      <c r="F54" s="6" t="n"/>
       <c r="G54" s="2" t="n"/>
     </row>
     <row r="55">
@@ -1912,13 +1941,13 @@
           <t>🌍 I already have insurance in the Netherlands. Do I still have to take out health insurance in Germany?</t>
         </is>
       </c>
-      <c r="D55" s="5" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>لدي تأمين في هولندا بالفعل. هل يجب عليّ مع ذلك الاشتراك في تأمين صحي في ألمانيا؟</t>
         </is>
       </c>
       <c r="E55" s="2" t="n"/>
-      <c r="F55" s="5" t="n"/>
+      <c r="F55" s="6" t="n"/>
       <c r="G55" s="2" t="n"/>
     </row>
     <row r="56">
@@ -1935,13 +1964,13 @@
           <t>Is the Rundfunkbeitrag a tax? Do I have to pay it?</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="D56" s="6" t="inlineStr">
         <is>
           <t>هل رسوم الـ GEZ ضريبة؟ وهل يجب أن أدفعها؟</t>
         </is>
       </c>
       <c r="E56" s="2" t="n"/>
-      <c r="F56" s="5" t="n"/>
+      <c r="F56" s="6" t="n"/>
       <c r="G56" s="2" t="n"/>
     </row>
     <row r="57">
@@ -1958,13 +1987,13 @@
           <t>My salary is 50,000 euros a year. Exactly how much tax will I pay?</t>
         </is>
       </c>
-      <c r="D57" s="5" t="inlineStr">
+      <c r="D57" s="6" t="inlineStr">
         <is>
           <t>راتبي السنوي 50,000 يورو. كم ستكون الضريبة التي سأدفعها بالضبط؟</t>
         </is>
       </c>
       <c r="E57" s="2" t="n"/>
-      <c r="F57" s="5" t="n"/>
+      <c r="F57" s="6" t="n"/>
       <c r="G57" s="2" t="n"/>
     </row>
     <row r="58">
@@ -1981,13 +2010,13 @@
           <t>The tax office made a decision that seems wrong to me, and I want to object. Will I win?</t>
         </is>
       </c>
-      <c r="D58" s="5" t="inlineStr">
+      <c r="D58" s="6" t="inlineStr">
         <is>
           <t>أصدرت مصلحة الضرائب قراراً يبدو لي خاطئاً وأريد الاعتراض عليه. هل سأربح؟</t>
         </is>
       </c>
       <c r="E58" s="2" t="n"/>
-      <c r="F58" s="5" t="n"/>
+      <c r="F58" s="6" t="n"/>
       <c r="G58" s="2" t="n"/>
     </row>
     <row r="59">
@@ -2004,13 +2033,13 @@
           <t>🌍 I'm Taiwanese and I'm here on a working holiday visa. I've been offered a permanent full-time job. Can I change my visa?</t>
         </is>
       </c>
-      <c r="D59" s="5" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>أنا تايواني وموجود هنا بتأشيرة عطلة العمل (Working Holiday). تلقيت عرض عمل ثابت بدوام كامل. هل يمكنني تغيير تأشيرتي؟</t>
         </is>
       </c>
       <c r="E59" s="2" t="n"/>
-      <c r="F59" s="5" t="n"/>
+      <c r="F59" s="6" t="n"/>
       <c r="G59" s="2" t="n"/>
     </row>
     <row r="60">
@@ -2027,13 +2056,13 @@
           <t>🌍 I'm Ukrainian. I worked for a German company for a year and was laid off. Can I get unemployment benefit?</t>
         </is>
       </c>
-      <c r="D60" s="5" t="inlineStr">
+      <c r="D60" s="6" t="inlineStr">
         <is>
           <t>أنا أوكراني، عملت لدى شركة ألمانية لمدة سنة ثم فُصلت من العمل. هل يمكنني الحصول على إعانة البطالة؟</t>
         </is>
       </c>
       <c r="E60" s="2" t="n"/>
-      <c r="F60" s="5" t="n"/>
+      <c r="F60" s="6" t="n"/>
       <c r="G60" s="2" t="n"/>
     </row>
     <row r="61">
@@ -2050,13 +2079,13 @@
           <t>🌍 I'm French and work in Germany. Can my American spouse live in Germany with me? Do they need a separate residence permit?</t>
         </is>
       </c>
-      <c r="D61" s="5" t="inlineStr">
+      <c r="D61" s="6" t="inlineStr">
         <is>
           <t>أنا فرنسي وأعمل في ألمانيا. هل يمكن لزوجتي أو زوجي الأمريكي العيش معي في ألمانيا؟ وهل يحتاج إلى تصريح إقامة خاص؟</t>
         </is>
       </c>
       <c r="E61" s="2" t="n"/>
-      <c r="F61" s="5" t="n"/>
+      <c r="F61" s="6" t="n"/>
       <c r="G61" s="2" t="n"/>
     </row>
   </sheetData>
@@ -2086,34 +2115,34 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Term in the questions</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>German original (for you)</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>OK?</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>Correction</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>البطاقة الزرقاء</t>
         </is>
@@ -2125,7 +2154,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>أوسبيلدونغ</t>
         </is>
@@ -2137,7 +2166,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>الإقامة الدائمة</t>
         </is>
@@ -2149,7 +2178,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>دائرة الأجانب</t>
         </is>
@@ -2161,7 +2190,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>الوكالة الاتحادية للعمل</t>
         </is>
@@ -2173,7 +2202,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>بطاقة الفرص</t>
         </is>
@@ -2185,7 +2214,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>أوبير</t>
         </is>
@@ -2197,7 +2226,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>تسجيل السكن</t>
         </is>
@@ -2209,7 +2238,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>إقامة البحث عن شغل / عمل</t>
         </is>
@@ -2221,7 +2250,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Working Holiday</t>
         </is>
@@ -2233,7 +2262,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>التأمين الاجتماعي للفنانين</t>
         </is>
@@ -2245,7 +2274,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Werkstudent / HiWi</t>
         </is>
@@ -2257,7 +2286,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>الميني جوب</t>
         </is>
@@ -2269,7 +2298,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>الكيندرغيلد</t>
         </is>
@@ -2281,7 +2310,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>الرقم الضريبي</t>
         </is>
@@ -2293,7 +2322,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>رسوم الـ GEZ</t>
         </is>
@@ -2305,7 +2334,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>إلغاء تسجيل السكن</t>
         </is>
@@ -2317,7 +2346,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>إعانة البطالة</t>
         </is>

</xml_diff>